<commit_message>
demo-kit: add guidance to the MSP CS sample '9. Links' tab
The single-column VE/VR link tables had empty example cells; add a
side-column instruction to type the imported VE study / VR track codes
under each header (code cells left empty so a typed code is always read
on import). No behaviour change.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/demo-kit/ValueLifecycle-Sample-MSP-Managed-ITSM-CS-Intake.xlsx
+++ b/demo-kit/ValueLifecycle-Sample-MSP-Managed-ITSM-CS-Intake.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="107">
   <si>
     <t>Account / customer</t>
   </si>
@@ -333,14 +333,20 @@
     <t>VE study code</t>
   </si>
   <si>
+    <t>← After import, type the VE study code in the cell directly below (e.g. VE-2026-0xx), then re-import to link.</t>
+  </si>
+  <si>
     <t>VR track code</t>
+  </si>
+  <si>
+    <t>← After import, type the VR track code in the cell directly below (e.g. VR-2026-0xx), then re-import to link.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -354,6 +360,10 @@
     <font>
       <b/>
       <color rgb="FFFFFFFF"/>
+    </font>
+    <font>
+      <i/>
+      <color rgb="FF6E685C"/>
     </font>
   </fonts>
   <fills count="3">
@@ -381,7 +391,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -389,6 +399,7 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -801,7 +812,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -840,7 +851,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -955,7 +966,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -1073,7 +1084,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -1144,7 +1155,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -1231,7 +1242,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -1294,7 +1305,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -1333,30 +1344,37 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A4"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
+    <col min="3" max="3" width="64" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="4" spans="1:1" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C1" s="5" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>104</v>
+        <v>105</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>106</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>